<commit_message>
cli: Implement e-certificate generation functionality with CLI support and Excel integration
</commit_message>
<xml_diff>
--- a/input/data.xlsx
+++ b/input/data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="X:\git-projects\e-certificate-generator\input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A285F322-0C06-4FC5-B497-D437B0998B39}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B6FC64A-B72D-417B-8BA6-C8E3D60EE922}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="15675" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
   <si>
     <t>Name</t>
   </si>
@@ -35,16 +35,39 @@
   </si>
   <si>
     <t>Ramya Krishnan</t>
+  </si>
+  <si>
+    <t>email</t>
+  </si>
+  <si>
+    <t>trisha@gmail.com</t>
+  </si>
+  <si>
+    <t>nayanthara@gmail.com</t>
+  </si>
+  <si>
+    <t>asin@gmail.com</t>
+  </si>
+  <si>
+    <t>ramya@gmail.com</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -67,13 +90,16 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -374,35 +400,59 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:A5"/>
+  <dimension ref="A1:B5"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <cols>
+    <col min="1" max="1" width="23.53125" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A1" t="s">
         <v>0</v>
       </c>
+      <c r="B1" t="s">
+        <v>5</v>
+      </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
         <v>1</v>
       </c>
+      <c r="B2" s="1" t="s">
+        <v>6</v>
+      </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
         <v>2</v>
       </c>
+      <c r="B3" s="1" t="s">
+        <v>7</v>
+      </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
         <v>3</v>
       </c>
+      <c r="B4" s="1" t="s">
+        <v>8</v>
+      </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
         <v>4</v>
       </c>
+      <c r="B5" s="1" t="s">
+        <v>9</v>
+      </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="B2" r:id="rId1" xr:uid="{1A3170EF-4E16-429B-A755-B14EFDE56680}"/>
+    <hyperlink ref="B3" r:id="rId2" xr:uid="{BCFE56BB-051C-4941-9281-4B653A7A6E2C}"/>
+    <hyperlink ref="B4" r:id="rId3" xr:uid="{4D92AD7E-7EC9-465F-8BB5-71BE0D2855BB}"/>
+    <hyperlink ref="B5" r:id="rId4" xr:uid="{ABC1E672-E56A-4E4C-B5F1-DA05E2F798FE}"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>